<commit_message>
wip C-013: case-flipping sort and search values, an error cell in the fixture, the header toggle dropping a sort, the scroll to a far match, semicolon and pipe named
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/book.xlsx
+++ b/tests/fixtures/book.xlsx
@@ -489,6 +489,10 @@
         <f>SUM(C2:C4)</f>
         <v>16.25</v>
       </c>
+      <c r="F5" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">

</xml_diff>